<commit_message>
structure of Excel Function
</commit_message>
<xml_diff>
--- a/excel/excel-101/OrderOfOperation-01.xlsx
+++ b/excel/excel-101/OrderOfOperation-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57de5c48f32aaca3/OfficeNewb/Videos/MicrosoftOffice/Excel2013MasterCourse/Exercises/New Exercises Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raj Khare\Raj\Udemy\ms-office\excel\excel-101\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{54B38A8E-5676-49A5-B3E9-6A4A5EC316B8}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{5475B79F-4326-4C20-8829-3614BD65926F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB84DE3E-7975-4ECA-A4BD-302AD739DCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="11040" xr2:uid="{2BB6ADC6-5ED7-4C10-85F5-FFCBA3ECC0D6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2BB6ADC6-5ED7-4C10-85F5-FFCBA3ECC0D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -138,21 +138,21 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -470,62 +470,68 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA501C94-4F54-4E06-95BD-06B20A90AD11}">
   <dimension ref="B2:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.26953125" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="3" t="s">
+      <c r="C2" s="8"/>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1">
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="5" t="s">
+    <row r="6" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="6" t="s">
+      <c r="C6" s="3">
+        <f>C3+C4+C5</f>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>0.08</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="8"/>
+      <c r="C8" s="7">
+        <f>C6*(C7+1)</f>
+        <v>329.40000000000003</v>
+      </c>
       <c r="D8" s="1"/>
     </row>
   </sheetData>
@@ -533,5 +539,14 @@
     <mergeCell ref="B2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Confidential – Oracle Internal</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{a4de43ec-192a-49eb-8e54-baeb8c71bbbe}" enabled="1" method="Standard" siteId="{4e2c6054-71cb-48f1-bd6c-3a9705aca71b}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>